<commit_message>
fix: harden local AI classification output
</commit_message>
<xml_diff>
--- a/output/requests.xlsx
+++ b/output/requests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -866,47 +866,47 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>065e312e-13cd-4b30-a4d2-56048b37d678</t>
+          <t>9ded455a-b942-4602-a4dc-980ec198790f</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-16T17:40:17.900524+00:00</t>
+          <t>2026-10-16T17:42:06.221541+00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Company Name</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Customer Company</t>
+          <t>Company ABC</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>example@company.com</t>
+          <t>johndoe@companyabc.com</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>clean and deduplicate csv export</t>
+          <t>data_cleanup</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Request to clean and deduplicate customer CSV export, fix missing columns, prepare an Excel file for the sales team.</t>
+          <t>CSV Export Clean-Up &amp; Preparation</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Review request</t>
+          <t>prepare an Excel file for the sales team</t>
         </is>
       </c>
       <c r="J8" t="n">
@@ -919,7 +919,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Hello Company Name. High priority. We received your request: Request to clean and deduplicate customer CSV export, fix missing columns, prepare an Excel file for the sales team.. Next step: Review request.</t>
+          <t>Hello Unknown. We received your data cleanup request: CSV Export Clean-Up &amp; Preparation. Next step: prepare an Excel file for the sales team.</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -931,12 +931,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>f4516c0f-3084-4cec-8dae-9e923710da3a</t>
+          <t>13d48538-f6a7-4b07-b085-f19c0add988a</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-16T17:40:20.192499+00:00</t>
+          <t>2026-10-16T17:42:07.562146+00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -949,20 +949,19 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>api automation</t>
+          <t>general</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Capture incoming leads with validated email data, remove duplicates, and send qualified leads to CRM.</t>
+          <t>No summary provided</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -980,7 +979,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Hello Unknown. High priority. We received your request: Capture incoming leads with validated email data, remove duplicates, and send qualified leads to CRM.. Next step: Review request.</t>
+          <t>Hello Unknown. We received your request: No summary provided. Next step: Review request.</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -992,12 +991,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>211c6325-bb5f-47eb-96a7-4ca7cd24c802</t>
+          <t>fc917ed5-a943-4c75-9856-cbebd6351643</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-16T17:40:22.543156+00:00</t>
+          <t>2026-10-16T17:42:10.349681+00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1007,13 +1006,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
+          <t>Company Details</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Company Email</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>urgent</t>
+          <t>general</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1023,12 +1026,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>No summary provided</t>
+          <t>Daily Management Report Creation from Spreadsheets</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Build a daily management report from several spreadsheets and flag missing or inconsistent values before 9 AM.</t>
+          <t>Build a daily management report with missing or inconsistent values in several spreadsheets before 9 AM</t>
         </is>
       </c>
       <c r="J10" t="n">
@@ -1041,10 +1044,390 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Hello Unknown. High priority. We received your request: No summary provided. Next step: Build a daily management report from several spreadsheets and flag missing or inconsistent values before 9 AM..</t>
+          <t>Hello Unknown. High priority. We received your request: Daily Management Report Creation from Spreadsheets. Next step: Build a daily management report with missing or inconsistent values in several spreadsheets before 9 AM.</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>f8982786-c86d-4ecc-a5fd-4c4bff89de90</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-10-16T17:42:50.353295+00:00</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>unknown@example.com</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>data_cleanup</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Need to clean and deduplicate customer CSV export, fix missing columns, and prepare an Excel file for the sales team.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Execute the specified actions.</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>demo-local</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Hello Unknown. High priority. We received your data cleanup request: Need to clean and deduplicate customer CSV export, fix missing columns, and prepare an Excel file for the sales team.. Next step: Execute the specified actions..</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>7655441a-20f3-4f1e-b532-3b196a8c93ca</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-10-16T17:42:52.379740+00:00</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>automation</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>API automation for lead capture, validation, deduplication, and delivery</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Create</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>demo-local</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Hello Unknown. High priority. We received your automation request: API automation for lead capture, validation, deduplication, and delivery. Next step: Create.</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>93d5143f-78bb-46c5-a82b-91b575585c19</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-10-16T17:42:54.860130+00:00</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>reporting</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>urgent</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Build a Daily Management Report From Several Spreadsheets and Flag Missing or Inconsistent Values Before 9 AM</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Review request</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>demo-local</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Hello Unknown. High priority. We received your reporting request: Build a Daily Management Report From Several Spreadsheets and Flag Missing or Inconsistent Values Before 9 AM. Next step: Review request.</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>33890352-d87c-476e-a94a-5747b93acfc3</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-10-16T17:43:23.112975+00:00</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>example_company</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>example@example.com</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>data_cleanup</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Request to clean and deduplicate customer CSV export, fix missing columns.</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Review request</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>demo-local</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Hello Unknown. We received your data cleanup request: Request to clean and deduplicate customer CSV export, fix missing columns.. Next step: Review request.</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>af2c80fb-eb69-418f-9f2b-8e42378f15a8</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-10-16T17:43:25.630378+00:00</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Example Company</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>johndoe@example.com</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>automation</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Capture incoming leads, validate email data, remove duplicates, and send qualified leads to CRM.</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>automation</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>demo-local</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Hello Unknown. High priority. We received your automation request: Capture incoming leads, validate email data, remove duplicates, and send qualified leads to CRM.. Next step: automation.</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>c5d763c9-f1ea-4ed7-b181-f4f5a17e494e</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-10-16T17:43:28.690760+00:00</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>user@example.com</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>reporting</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>urgent</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Daily Management Report from Spreadsheets: Flagging Missing or Inconsistent Values Before 9 AM</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>build a daily management report from several spreadsheets and flag missing or inconsistent values before 9 AM</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>demo-local</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Hello User. High priority. We received your reporting request: Daily Management Report from Spreadsheets: Flagging Missing or Inconsistent Values Before 9 AM. Next step: build a daily management report from several spreadsheets and flag missing or inconsistent values before 9 AM.</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
         <is>
           <t>processed</t>
         </is>

</xml_diff>